<commit_message>
docs(plans): add year-plan indicators plan
</commit_message>
<xml_diff>
--- a/plans/reports/261007-doi-chieu-cot-ke-hoach-file-voi-phan-mem.xlsx
+++ b/plans/reports/261007-doi-chieu-cot-ke-hoach-file-voi-phan-mem.xlsx
@@ -1413,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1436,14 +1436,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>19 cột của file gộp còn 13 chỉ tiêu: 4 đã có, 9 thêm mới. Nhượng quyền không là chỉ tiêu riêng, số cộng vào khai thác.</t>
+          <t>19 cột của file gộp còn 15 chỉ tiêu: 4 đã có, 11 thêm mới. Nhượng quyền không là chỉ tiêu riêng, số cộng vào khai thác. Hàng hóa tách khỏi thu mua ở tiêu thụ và doanh thu. Tồn kho thành phẩm và hợp đồng xem tab «Kế hoạch final».</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>A. Chỉ tiêu sau khi gộp (13 chỉ tiêu)</t>
+          <t>A. Chỉ tiêu lấy từ file sau khi gộp (15 chỉ tiêu)</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Tiêu thụ thu mua (gồm thành phẩm mua thêm)</t>
+          <t>Tiêu thụ thu mua</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R − J</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tách hàng hóa khỏi R (ước tính)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Tiêu thụ tổng</t>
+          <t>Tiêu thụ hàng hóa</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Bằng dòng 8 + dòng 9</t>
+          <t>Coi hàng hóa mua về bán hết trong năm (ước tính)</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Tự cộng</t>
+          <t>Nhập</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -1895,32 +1895,32 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Doanh thu</t>
+          <t>Tiêu thụ</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Doanh thu khai thác</t>
+          <t>Tiêu thụ tổng</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>tỷ đồng</t>
+          <t>tấn</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>T  (U + V)</t>
+          <t>O</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Gồm tự khai thác + nhượng quyền; chia 1.000</t>
+          <t>Bằng dòng 8 + 9 + 10</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Nhập</t>
+          <t>Tự cộng</t>
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Doanh thu thu mua (gồm hàng hóa)</t>
+          <t>Doanh thu khai thác</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T  (U + V)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Chia 1.000</t>
+          <t>Gồm tự khai thác + nhượng quyền; chia 1.000</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1978,154 +1978,170 @@
           <t>Doanh thu</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Doanh thu thu mua</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>tỷ đồng</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>W × (R − J) ÷ R</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Chia W theo tỷ lệ tấn (ước tính); chia 1.000</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Doanh thu</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Doanh thu hàng hóa</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>tỷ đồng</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>W × J ÷ R</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Như trên</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Doanh thu</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Kế hoạch doanh thu (tổng)</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>tỷ đồng</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Bằng dòng 11 + dòng 12; chia 1.000</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Bằng dòng 12 + 13 + 14; chia 1.000</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Tự cộng</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>Đã có</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>B. Cột file không còn là chỉ tiêu riêng (6 cột, đều gộp vào khai thác)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Cột trong file</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Nhóm</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Tên cột trong file</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Đơn vị</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Gộp vào dòng</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Khai thác</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>SL tự khai thác</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>tấn</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Đã nằm trong E</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Khai thác</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>SL nhượng quyền</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>tấn</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>4 công ty có số, tổng 1.627 tấn (xem mục C)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Chế biến</t>
+          <t>Khai thác</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Chế biến nhượng quyền</t>
+          <t>SL tự khai thác</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2135,29 +2151,29 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Toàn bộ bằng 0</t>
+          <t>Đã nằm trong E</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Tiêu thụ</t>
+          <t>Khai thác</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Tiêu thụ NQ</t>
+          <t>SL nhượng quyền</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2167,272 +2183,304 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Toàn bộ bằng 0</t>
+          <t>4 công ty có số, tổng 1.627 tấn (xem mục C)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Doanh thu</t>
+          <t>Chế biến</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>DT mủ tự KT</t>
+          <t>Chế biến nhượng quyền</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>triệu đồng</t>
+          <t>tấn</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Đã nằm trong T</t>
+          <t>Toàn bộ bằng 0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Tiêu thụ</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Tiêu thụ NQ</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Toàn bộ bằng 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Doanh thu</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>DT mủ tự KT</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>triệu đồng</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Đã nằm trong T</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
           <t>V</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Doanh thu</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>DT mủ NQ</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>triệu đồng</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>4 công ty có số, tổng 255,1 tỷ (xem mục C)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>C. Công ty có nhượng quyền (số cộng vào khai thác)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="42" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>TT</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr"/>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Công ty</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>SL nhượng quyền (tấn)</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>DT nhượng quyền (tỷ đồng)</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>KH khai thác sau gộp (tấn)</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>CS Dầu Tiếng</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="13" t="n">
-        <v>890</v>
-      </c>
-      <c r="F31" s="14" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="13" t="n">
-        <v>25840</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>CS Lộc Ninh</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="14" t="n">
-        <v>238.8</v>
-      </c>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="13" t="n">
-        <v>32300</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B33" s="5" t="n"/>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>CP CS Tân Biên</t>
+          <t>CS Dầu Tiếng</t>
         </is>
       </c>
       <c r="D33" s="5" t="n"/>
       <c r="E33" s="13" t="n">
-        <v>80</v>
+        <v>890</v>
       </c>
       <c r="F33" s="14" t="n">
-        <v>1.1</v>
+        <v>9.6</v>
       </c>
       <c r="G33" s="5" t="n"/>
       <c r="H33" s="13" t="n">
-        <v>3550</v>
+        <v>25840</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B34" s="5" t="n"/>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>CP CS Tây Ninh</t>
+          <t>CS Lộc Ninh</t>
         </is>
       </c>
       <c r="D34" s="5" t="n"/>
       <c r="E34" s="13" t="n">
-        <v>357</v>
+        <v>0</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>5.6</v>
+        <v>238.8</v>
       </c>
       <c r="G34" s="5" t="n"/>
       <c r="H34" s="13" t="n">
-        <v>9400</v>
+        <v>32300</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B35" s="5" t="n"/>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>CS Chư prông</t>
+          <t>CP CS Tân Biên</t>
         </is>
       </c>
       <c r="D35" s="5" t="n"/>
       <c r="E35" s="13" t="n">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="F35" s="14" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="G35" s="5" t="n"/>
       <c r="H35" s="13" t="n">
+        <v>3550</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>CP CS Tây Ninh</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="13" t="n">
+        <v>357</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="13" t="n">
+        <v>9400</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>CS Chư prông</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="13" t="n">
         <v>13950</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>D. Cần anh chốt</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="4" t="n">
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>KH doanh thu lấy cột S («DT tổng» 26.936 tỷ) hay «DT bán hàng» dòng 57 (27.902 tỷ)?</t>
-        </is>
-      </c>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="16" t="n"/>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Ô «KH tiêu thụ HĐ chuyến» đang có: giữ song song với 3 ô tiêu thụ mới, hay thay bằng 3 ô mới?</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="15" t="n"/>
-      <c r="G39" s="15" t="n"/>
-      <c r="H39" s="16" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>4 ô tổng (thu mua, chế biến, tiêu thụ, doanh thu) em để TỰ CỘNG từ chi tiết, đơn vị chỉ nhập chi tiết. Riêng ô «KH doanh thu» đang nhập tay sẽ chuyển sang tự cộng. Đồng ý không?</t>
         </is>
       </c>
       <c r="C40" s="15" t="n"/>
@@ -2442,11 +2490,94 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="16" t="n"/>
     </row>
+    <row r="41" ht="15" customHeight="1">
+      <c r="A41" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Ô «KH tiêu thụ HĐ chuyến» đang có: giữ song song với 4 ô tiêu thụ mới, hay thay bằng 4 ô mới?</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="15" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="15" t="n"/>
+      <c r="H41" s="16" t="n"/>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>5 ô tổng (thu mua, chế biến, tiêu thụ, doanh thu, tồn kho) để TỰ CỘNG từ chi tiết; ô «KH doanh thu» đang nhập tay sẽ chuyển sang tự cộng. Đồng ý không?</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="16" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Tiêu thụ hàng hóa = J (coi mua về bán hết trong năm), tiêu thụ thu mua = R − J. Trong file 56/63 công ty có R − N = J, khớp cách hiểu này. Đồng ý không?</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="15" t="n"/>
+      <c r="G43" s="15" t="n"/>
+      <c r="H43" s="16" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>File không tách doanh thu thu mua / hàng hóa: tạm chia W theo tỷ lệ tấn, hay nhờ Ban bổ sung số thật?</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="15" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="15" t="n"/>
+      <c r="H44" s="16" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>KH tồn kho thành phẩm (khai thác / thu mua / hàng hóa): tính tại 31/12? Ban hay đơn vị nhập? Phần mềm chưa khai tồn kho theo nguồn nên chưa có số thực hiện để so.</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="15" t="n"/>
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="15" t="n"/>
+      <c r="H45" s="16" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B38:H38"/>
+  <mergeCells count="6">
     <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B39:H39"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="B43:H43"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B45:H45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2459,17 +2590,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2482,7 +2613,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>6 nhóm · 17 chỉ tiêu: 8 đã có trên phần mềm, 9 thêm mới. Mỗi dòng là một ô trên màn Kế hoạch năm.</t>
+          <t>7 nhóm · 23 chỉ tiêu: 8 đã có trên phần mềm, 15 thêm mới. Mỗi dòng là một ô trên màn Kế hoạch năm.</t>
         </is>
       </c>
     </row>
@@ -2812,14 +2943,14 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="33" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="17" t="n"/>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Tiêu thụ thu mua (gồm thành phẩm mua thêm)</t>
+          <t>Tiêu thụ thu mua</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -2829,7 +2960,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R − J</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -2842,16 +2973,20 @@
           <t>Thêm mới</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Ước tính: file chỉ có R (thu mua gồm hàng hóa), trừ phần hàng hóa J</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="18" t="n"/>
+      <c r="B14" s="17" t="n"/>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Tiêu thụ tổng</t>
+          <t>Tiêu thụ hàng hóa</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -2861,12 +2996,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>O  (= P + R)</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Tự cộng</t>
+          <t>Nhập</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -2874,35 +3009,35 @@
           <t>Thêm mới</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Ước tính: coi hàng hóa mua về bán hết trong năm</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Doanh thu</t>
-        </is>
-      </c>
+      <c r="B15" s="18" t="n"/>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Doanh thu khai thác</t>
+          <t>Tiêu thụ tổng</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>tỷ đồng</t>
+          <t>tấn</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>T  (= U + V)</t>
+          <t>O  (= P + R)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Nhập</t>
+          <t>Tự cộng</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -2910,20 +3045,20 @@
           <t>Thêm mới</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Gồm cả nhượng quyền; file tính triệu đồng, chia 1.000</t>
-        </is>
-      </c>
+      <c r="H15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="17" t="n"/>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Doanh thu</t>
+        </is>
+      </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Doanh thu thu mua (gồm hàng hóa)</t>
+          <t>Doanh thu khai thác</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2933,7 +3068,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T  (= U + V)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -2948,7 +3083,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Chia 1.000</t>
+          <t>Gồm cả nhượng quyền; file tính triệu đồng, chia 1.000</t>
         </is>
       </c>
     </row>
@@ -2956,10 +3091,10 @@
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Kế hoạch doanh thu (tổng)</t>
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Doanh thu thu mua</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2969,22 +3104,22 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>S  (= T + W)</t>
+          <t>W × (R − J) ÷ R</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Tự cộng</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Đã có</t>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Ô hiện nhập tay, chuyển sang tự cộng</t>
+          <t>Ước tính: file không tách hàng hóa, tạm chia W theo tỷ lệ tấn</t>
         </is>
       </c>
     </row>
@@ -2992,25 +3127,20 @@
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Hợp đồng
-(đơn vị tự khai)</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Kế hoạch tiêu thụ — HĐ chuyến</t>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Doanh thu hàng hóa</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>tấn</t>
+          <t>tỷ đồng</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>— (file không có)</t>
+          <t>W × J ÷ R</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -3018,14 +3148,14 @@
           <t>Nhập</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Đã có</t>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Chờ anh chốt: giữ hay thay bằng 3 ô tiêu thụ</t>
+          <t>Như trên</t>
         </is>
       </c>
     </row>
@@ -3033,25 +3163,25 @@
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="17" t="n"/>
+      <c r="B19" s="18" t="n"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>HĐ dài hạn đã ký</t>
+          <t>Kế hoạch doanh thu (tổng)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>tấn</t>
+          <t>tỷ đồng</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>— (file không có)</t>
+          <t>S  (= T + W)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Nhập</t>
+          <t>Tự cộng</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -3059,16 +3189,24 @@
           <t>Đã có</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Ô hiện nhập tay, chuyển sang tự cộng</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="33" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>HĐ dài hạn năm trước chuyển sang</t>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Tồn kho thành phẩm</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Kế hoạch tồn kho thành phẩm — khai thác</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -3086,69 +3224,287 @@
           <t>Nhập</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Đã có</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Số thời điểm. Phần mềm chưa khai tồn kho theo nguồn nên chưa có số thực hiện để so</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Kế hoạch tồn kho thành phẩm — thu mua</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Như trên</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Kế hoạch tồn kho thành phẩm — hàng hóa</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Như trên</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Kế hoạch tồn kho thành phẩm — tổng</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Tự cộng</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Bằng khai thác + thu mua + hàng hóa</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Hợp đồng
+(đơn vị tự khai)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Kế hoạch tiêu thụ — HĐ chuyến</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Đã có</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Chờ anh chốt: giữ hay thay bằng 4 ô tiêu thụ ở trên</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>HĐ dài hạn đã ký</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đã có</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>HĐ dài hạn năm trước chuyển sang</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Đã có</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>HĐ chuyến năm trước chuyển sang</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>tấn</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>— (file không có)</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Nhập</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>Đã có</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Cộng: 6 nhóm</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>17 chỉ tiêu</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="19" t="n"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
+      <c r="H27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Cộng: 7 nhóm</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>23 chỉ tiêu</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
+      <c r="H28" s="19" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B15:B17"/>
+  <mergeCells count="6">
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B12:B15"/>
     <mergeCell ref="B9:B11"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B16:B19"/>
     <mergeCell ref="B6:B8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(plans): add contract totals to year-plan docs
</commit_message>
<xml_diff>
--- a/plans/reports/261007-doi-chieu-cot-ke-hoach-file-voi-phan-mem.xlsx
+++ b/plans/reports/261007-doi-chieu-cot-ke-hoach-file-voi-phan-mem.xlsx
@@ -1440,6 +1440,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -2089,6 +2090,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -2320,6 +2322,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
@@ -2467,6 +2470,7 @@
         <v>13950</v>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
@@ -2512,7 +2516,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>5 ô tổng (thu mua, chế biến, tiêu thụ, doanh thu, tồn kho) để TỰ CỘNG từ chi tiết; ô «KH doanh thu» đang nhập tay sẽ chuyển sang tự cộng. Đồng ý không?</t>
+          <t>7 ô tổng (thu mua, chế biến, tiêu thụ, doanh thu, tồn kho, HĐ dài hạn, HĐ chuyến) để TỰ CỘNG từ chi tiết; ô «KH doanh thu» đang nhập tay sẽ chuyển sang tự cộng. Đồng ý không?</t>
         </is>
       </c>
       <c r="C42" s="15" t="n"/>
@@ -2588,9 +2592,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2613,7 +2617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>7 nhóm · 23 chỉ tiêu: 8 đã có trên phần mềm, 15 thêm mới. Mỗi dòng là một ô trên màn Kế hoạch năm.</t>
+          <t>7 nhóm · 25 chỉ tiêu: 8 đã có trên phần mềm, 17 thêm mới. Mỗi dòng là một ô trên màn Kế hoạch năm.</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3359,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Kế hoạch tiêu thụ — HĐ chuyến</t>
+          <t>HĐ dài hạn đã ký</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -3378,11 +3382,7 @@
           <t>Đã có</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Chờ anh chốt: giữ hay thay bằng 4 ô tiêu thụ ở trên</t>
-        </is>
-      </c>
+      <c r="H24" s="5" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="n">
@@ -3391,7 +3391,7 @@
       <c r="B25" s="17" t="n"/>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>HĐ dài hạn đã ký</t>
+          <t>HĐ dài hạn năm trước chuyển sang</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -3421,9 +3421,9 @@
         <v>22</v>
       </c>
       <c r="B26" s="17" t="n"/>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>HĐ dài hạn năm trước chuyển sang</t>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Tổng HĐ dài hạn thực hiện trong năm</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -3438,74 +3438,150 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Nhập</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>Đã có</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr"/>
+          <t>Tự cộng</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Bằng 2 dòng trên</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="18" t="n"/>
+      <c r="B27" s="17" t="n"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
+          <t>Kế hoạch tiêu thụ — HĐ chuyến</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Nhập</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Đã có</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Chờ anh chốt: giữ hay thay bằng 4 ô tiêu thụ ở trên</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
           <t>HĐ chuyến năm trước chuyển sang</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>tấn</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>— (file không có)</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Nhập</t>
         </is>
       </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>Đã có</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Tổng HĐ chuyến thực hiện trong năm</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>— (file không có)</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Tự cộng</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Thêm mới</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Bằng 2 dòng trên</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>Cộng: 7 nhóm</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr">
-        <is>
-          <t>23 chỉ tiêu</t>
-        </is>
-      </c>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="19" t="n"/>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="19" t="n"/>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>25 chỉ tiêu</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="B12:B15"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B24:B27"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B24:B29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>